<commit_message>
feat: add resource dimension linting
</commit_message>
<xml_diff>
--- a/data-tables/Datas/resources.xlsx
+++ b/data-tables/Datas/resources.xlsx
@@ -434,12 +434,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,6 +459,11 @@
           <t>name</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -475,6 +481,11 @@
           <t>display name</t>
         </is>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>quantity dimension</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -488,6 +499,11 @@
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
@@ -505,6 +521,11 @@
           <t>Fish</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>fish</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
@@ -516,6 +537,11 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>Prestige Point</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>prestige</t>
         </is>
       </c>
     </row>

</xml_diff>